<commit_message>
modifica JoinSoft in Joinsoft
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#JOINSOFTSRLXX/Joinsoft_Srl/Gestione_Stabilimenti_Termali/Ver_6.31/report-checklist.xlsx
+++ b/GATEWAY/S1#111#JOINSOFTSRLXX/Joinsoft_Srl/Gestione_Stabilimenti_Termali/Ver_6.31/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francesco\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191072ED-FCC0-4F08-A4D2-44197A81C0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C71ACE-9B70-465E-84F3-E7505B14DD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="-13620" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -2179,9 +2179,6 @@
     <t>subject_application_id: Gestione_Stabilimenti_Termali</t>
   </si>
   <si>
-    <t>subject_application_vendor:JoinSoft_Srl</t>
-  </si>
-  <si>
     <t>subject_application_version:Ver_6.31</t>
   </si>
   <si>
@@ -2243,6 +2240,9 @@
   </si>
   <si>
     <t>2191dcd5e052e59d873f96feb5ac1f20</t>
+  </si>
+  <si>
+    <t>subject_application_vendor:Joinsoft_Srl</t>
   </si>
 </sst>
 </file>
@@ -4428,7 +4428,7 @@
       <c r="A4" s="57"/>
       <c r="B4" s="58"/>
       <c r="C4" s="61" t="s">
-        <v>590</v>
+        <v>611</v>
       </c>
       <c r="D4" s="53"/>
       <c r="E4" s="4"/>
@@ -4455,7 +4455,7 @@
       <c r="A5" s="59"/>
       <c r="B5" s="60"/>
       <c r="C5" s="61" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D5" s="53"/>
       <c r="F5" s="6"/>
@@ -4806,10 +4806,10 @@
         <v>46099</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="I14" s="42" t="s">
         <v>439</v>
@@ -4867,10 +4867,10 @@
         <v>46099</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="H15" s="37" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="I15" s="42" t="s">
         <v>439</v>
@@ -5186,10 +5186,10 @@
         <v>46099</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="I22" s="42" t="s">
         <v>439</v>
@@ -5247,10 +5247,10 @@
         <v>46099</v>
       </c>
       <c r="G23" s="37" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="H23" s="37" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="I23" s="42" t="s">
         <v>439</v>
@@ -12016,13 +12016,13 @@
         <v>46087</v>
       </c>
       <c r="G164" s="37" t="s">
+        <v>591</v>
+      </c>
+      <c r="H164" s="37" t="s">
         <v>592</v>
       </c>
-      <c r="H164" s="37" t="s">
+      <c r="I164" s="42" t="s">
         <v>593</v>
-      </c>
-      <c r="I164" s="42" t="s">
-        <v>594</v>
       </c>
       <c r="J164" s="38" t="s">
         <v>64</v>
@@ -12063,13 +12063,13 @@
         <v>46087</v>
       </c>
       <c r="G165" s="37" t="s">
+        <v>594</v>
+      </c>
+      <c r="H165" s="37" t="s">
         <v>595</v>
       </c>
-      <c r="H165" s="37" t="s">
+      <c r="I165" s="42" t="s">
         <v>596</v>
-      </c>
-      <c r="I165" s="42" t="s">
-        <v>597</v>
       </c>
       <c r="J165" s="38" t="s">
         <v>64</v>
@@ -13024,13 +13024,13 @@
         <v>46087</v>
       </c>
       <c r="G186" s="37" t="s">
+        <v>597</v>
+      </c>
+      <c r="H186" s="37" t="s">
         <v>598</v>
       </c>
-      <c r="H186" s="37" t="s">
+      <c r="I186" s="42" t="s">
         <v>599</v>
-      </c>
-      <c r="I186" s="42" t="s">
-        <v>600</v>
       </c>
       <c r="J186" s="38" t="s">
         <v>64</v>
@@ -13071,13 +13071,13 @@
         <v>46087</v>
       </c>
       <c r="G187" s="37" t="s">
+        <v>600</v>
+      </c>
+      <c r="H187" s="37" t="s">
         <v>601</v>
       </c>
-      <c r="H187" s="37" t="s">
+      <c r="I187" s="42" t="s">
         <v>602</v>
-      </c>
-      <c r="I187" s="42" t="s">
-        <v>603</v>
       </c>
       <c r="J187" s="38" t="s">
         <v>64</v>
@@ -19626,12 +19626,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19779,15 +19776,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -19811,18 +19820,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
per i test 449, 472 aggiornato WII
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#JOINSOFTSRLXX/Joinsoft_Srl/Gestione_Stabilimenti_Termali/Ver_6.31/report-checklist.xlsx
+++ b/GATEWAY/S1#111#JOINSOFTSRLXX/Joinsoft_Srl/Gestione_Stabilimenti_Termali/Ver_6.31/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francesco\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8D5D9A-1C9D-4C7C-86E7-063C459D49A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3BDD04-DC85-4022-BDF1-622FEB946ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="-13620" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -2218,15 +2218,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.0ab541df2fccb2d9ccd6c5af009ab97c1739337983a95b9f75c864f2b3be6d91.aaf3c21f15^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-25T08:16:24.491Z</t>
-  </si>
-  <si>
-    <t>12ebdfc2aebf6b8a6ebda2d147df9887</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.c14e8b1bfef36f6f2b3d891d73399882c9dc8bdaa9903a9d2190c18ebe8c50e3.853716450e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-25T08:16:25.323Z</t>
   </si>
   <si>
@@ -2236,13 +2227,22 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.9f8f38100155863f456fd3d087e733ce5ca0cc2821d2afd2d421e6634748b701.bdfff4f7ab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-25T08:16:26.114Z</t>
-  </si>
-  <si>
-    <t>b5330938e686802afba7197238e5832f</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.a6b7f56520b0f47b553d484c4e3b9f6b6dde76ca191e6da490ac9cdb89392068.674db9706a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-03-26T10:48:38.618Z</t>
+  </si>
+  <si>
+    <t>05bc761170cd807475bccbfad15d2f9b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.7cba0fe9ddcb13ec116289dec5aee787f34669b61f5c77579b24c014b72c3671.d249bf7896^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-26T10:48:37.517Z</t>
+  </si>
+  <si>
+    <t>95f5b589ea7dd17ed618b51746249d25</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.1564e1cd5a436803ffc2630cb90cde970aa196856e93241d1ab81e12533fbfba.524235aac1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -12043,7 +12043,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="35">
         <v>449</v>
       </c>
@@ -12060,16 +12060,16 @@
         <v>380</v>
       </c>
       <c r="F165" s="47">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="G165" s="37" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="H165" s="37" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="I165" s="42" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="J165" s="38" t="s">
         <v>64</v>
@@ -13024,13 +13024,13 @@
         <v>46106</v>
       </c>
       <c r="G186" s="37" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="H186" s="37" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="I186" s="42" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="J186" s="38" t="s">
         <v>64</v>
@@ -13051,7 +13051,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A187" s="35">
         <v>472</v>
       </c>
@@ -13068,16 +13068,16 @@
         <v>414</v>
       </c>
       <c r="F187" s="47">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="G187" s="37" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="H187" s="37" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="I187" s="42" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="J187" s="38" t="s">
         <v>64</v>
@@ -17352,7 +17352,7 @@
   <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="472"/>
+        <filter val="449"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -17371,7 +17371,7 @@
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>
@@ -19625,12 +19625,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19778,15 +19775,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -19810,18 +19819,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>